<commit_message>
chore: verify and package v0.1 candidate
</commit_message>
<xml_diff>
--- a/Evaluation-Template.xlsx
+++ b/Evaluation-Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R991e16a0cf674394"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batch" sheetId="2" r:id="R9adea415ec8b43d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R989c6a659a2c4501"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batch" sheetId="2" r:id="R14b078c666774795"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
fix: correct protocol gates and review workflow
</commit_message>
<xml_diff>
--- a/Evaluation-Template.xlsx
+++ b/Evaluation-Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R989c6a659a2c4501"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batch" sheetId="2" r:id="R14b078c666774795"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R33e190c6a5e24cb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batch" sheetId="2" r:id="R8a85d6d122fd4128"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -66,7 +66,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="14">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -102,6 +102,7 @@
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -360,7 +361,7 @@
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>One assessment per copy. v0.1 release candidate.</x:v>
+        <x:v>One assessment per copy. v0.1-rc.2; unvalidated method.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3"/>
@@ -463,7 +464,7 @@
         <x:v>Reference-set defect recall</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
-        <x:f>IF(COUNT(B26,B25)&lt;2,"Not evaluated",IF(OR(B26&lt;0,B25&lt;0,MOD(B26,1)&lt;&gt;0,MOD(B25,1)&lt;&gt;0,B26&gt;B25),"Invalid counts",IF(B25=0,"n.a.",B26/B25)))</x:f>
+        <x:f>IF(AND(COUNT(B25:B28)=4,OR(B27&gt;B25,B28&gt;B26,B26-B28&gt;B25-B27,B26&gt;B25,B28&gt;B27,MIN(B25:B28)&lt;0,MOD(B25,1)&lt;&gt;0,MOD(B26,1)&lt;&gt;0,MOD(B27,1)&lt;&gt;0,MOD(B28,1)&lt;&gt;0)),"Invalid counts",IF(COUNT(B26,B25)&lt;2,"Not evaluated",IF(OR(B26&lt;0,B25&lt;0,MOD(B26,1)&lt;&gt;0,MOD(B25,1)&lt;&gt;0,B26&gt;B25),"Invalid counts",IF(B25=0,"n.a.",B26/B25))))</x:f>
         <x:v>Not evaluated</x:v>
       </x:c>
       <x:c r="C14"/>
@@ -505,7 +506,7 @@
         <x:v>Omission recognition</x:v>
       </x:c>
       <x:c r="B17" s="7" t="str">
-        <x:f>IF(AND(ISNUMBER(B27),ISNUMBER(B25),B27&gt;B25),"Invalid counts",IF(AND(ISNUMBER(B28),ISNUMBER(B26),B28&gt;B26),"Invalid counts",IF(COUNT(B28,B27)&lt;2,"Not evaluated",IF(OR(B28&lt;0,B27&lt;0,MOD(B28,1)&lt;&gt;0,MOD(B27,1)&lt;&gt;0,B28&gt;B27),"Invalid counts",IF(B27=0,"n.a.",B28/B27)))))</x:f>
+        <x:f>IF(COUNT(B25:B28)&lt;4,"Not evaluated",IF(OR(B27&gt;B25,B28&gt;B26,B26-B28&gt;B25-B27,B26&gt;B25,B28&gt;B27,MIN(B25:B28)&lt;0,MOD(B25,1)&lt;&gt;0,MOD(B26,1)&lt;&gt;0,MOD(B27,1)&lt;&gt;0,MOD(B28,1)&lt;&gt;0),"Invalid counts",IF(COUNT(B28,B27)&lt;2,"Not evaluated",IF(OR(B28&lt;0,B27&lt;0,MOD(B28,1)&lt;&gt;0,MOD(B27,1)&lt;&gt;0,B28&gt;B27),"Invalid counts",IF(B27=0,"n.a.",B28/B27)))))</x:f>
         <x:v>Not evaluated</x:v>
       </x:c>
       <x:c r="C17"/>
@@ -547,7 +548,7 @@
         <x:v>Artifact disposition</x:v>
       </x:c>
       <x:c r="B20" s="11" t="str">
-        <x:f>IF(OR(B16="Invalid counts",B18="Invalid counts",AND(ISNUMBER(B33),OR(B33&lt;0,MOD(B33,1)&lt;&gt;0)),AND(ISNUMBER(B34),OR(B34&lt;0,MOD(B34,1)&lt;&gt;0))),"Invalid counts",IF(OR(AND(ISNUMBER(B33),B33&gt;0),AND(COUNT(B29:B30)=2,B30&lt;B29),AND(COUNT(B31:B32)=2,B32&lt;B31)),"Hold for remediation",IF(OR(B35="No",AND(ISNUMBER(B34),B34&gt;0),AND(ISNUMBER(B31),B31=0)),"Insufficient evidence",IF(OR(COUNT(B29:B34)&lt;6,B35&lt;&gt;"Yes"),"Not evaluated","Eligible for handoff review"))))</x:f>
+        <x:f>IF(OR(B16="Invalid counts",B18="Invalid counts",AND(ISNUMBER(B33),OR(B33&lt;0,MOD(B33,1)&lt;&gt;0)),AND(ISNUMBER(B34),OR(B34&lt;0,MOD(B34,1)&lt;&gt;0)),AND(ISNUMBER(B36),OR(B36&lt;0,MOD(B36,1)&lt;&gt;0))),"Invalid counts",IF(OR(COUNT(B29:B34,B36)&lt;7,AND(B35&lt;&gt;"Yes",B35&lt;&gt;"No")),"Not evaluated",IF(B30+B32+B34+B36&lt;&gt;B29+B31,"Invalid counts",IF(OR(B33&gt;0,B36&gt;0),"Hold for remediation",IF(OR(B34&gt;0,B35="No",B31=0),"Insufficient evidence","Eligible for handoff review")))))</x:f>
         <x:v>Not evaluated</x:v>
       </x:c>
       <x:c r="C20"/>
@@ -698,7 +699,7 @@
       <x:c r="B34" s="6"/>
       <x:c r="C34"/>
       <x:c r="D34" s="2" t="str">
-        <x:v>Count unassessed mandatory requirements and recovery items.</x:v>
+        <x:v>Unassessed requirement + recovery rows; disjoint from failed rows.</x:v>
       </x:c>
       <x:c r="E34" s="2"/>
     </x:row>
@@ -714,10 +715,14 @@
       <x:c r="E35" s="2"/>
     </x:row>
     <x:row r="36" ht="25" customHeight="1">
-      <x:c r="A36" s="2"/>
-      <x:c r="B36" s="2"/>
+      <x:c r="A36" s="2" t="str">
+        <x:v>Documented failed mandatory checks</x:v>
+      </x:c>
+      <x:c r="B36" s="6"/>
       <x:c r="C36"/>
-      <x:c r="D36" s="2"/>
+      <x:c r="D36" s="2" t="str">
+        <x:v>Verified + failed + unassessed must equal total required checks.</x:v>
+      </x:c>
       <x:c r="E36" s="2"/>
     </x:row>
     <x:row r="37" ht="25" customHeight="1">
@@ -745,7 +750,7 @@
   <x:conditionalFormatting sqref="B20:B20">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Hold"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="4">
+  <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="B9">
       <x:formula1>"Ready,Not ready,Unable to assess"</x:formula1>
     </x:dataValidation>
@@ -758,6 +763,9 @@
     </x:dataValidation>
     <x:dataValidation type="list" sqref="B35">
       <x:formula1>"Yes,No"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="B36">
+      <x:formula1>0</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -954,7 +962,7 @@
       <x:c r="D16" s="4"/>
       <x:c r="E16" s="4"/>
       <x:c r="F16" t="str">
-        <x:f>IF(COUNTA(A16:E16)=0,"",IF(OR(A16="",B16="",COUNTIFS($A$16:$A$35,A16)&gt;1,AND(C16&lt;&gt;"Ready",C16&lt;&gt;"Nonready",C16&lt;&gt;"Unknown"),AND(D16&lt;&gt;"Ready",D16&lt;&gt;"Not ready",D16&lt;&gt;"Unable to assess",D16&lt;&gt;"Missing",D16&lt;&gt;"")),"Invalid record",IF(B16&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A16:E16)=0,"",IF(OR(A16="",B16="",COUNTIFS($A$16:$A$35,A16)&gt;1,AND(C16&lt;&gt;"Ready",C16&lt;&gt;"Nonready",C16&lt;&gt;"Unknown"),AND(D16&lt;&gt;"Ready",D16&lt;&gt;"Not ready",D16&lt;&gt;"Unable to assess",D16&lt;&gt;"Missing",D16&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B16)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
@@ -964,7 +972,7 @@
       <x:c r="D17" s="4"/>
       <x:c r="E17" s="4"/>
       <x:c r="F17" t="str">
-        <x:f>IF(COUNTA(A17:E17)=0,"",IF(OR(A17="",B17="",COUNTIFS($A$16:$A$35,A17)&gt;1,AND(C17&lt;&gt;"Ready",C17&lt;&gt;"Nonready",C17&lt;&gt;"Unknown"),AND(D17&lt;&gt;"Ready",D17&lt;&gt;"Not ready",D17&lt;&gt;"Unable to assess",D17&lt;&gt;"Missing",D17&lt;&gt;"")),"Invalid record",IF(B17&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A17:E17)=0,"",IF(OR(A17="",B17="",COUNTIFS($A$16:$A$35,A17)&gt;1,AND(C17&lt;&gt;"Ready",C17&lt;&gt;"Nonready",C17&lt;&gt;"Unknown"),AND(D17&lt;&gt;"Ready",D17&lt;&gt;"Not ready",D17&lt;&gt;"Unable to assess",D17&lt;&gt;"Missing",D17&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B17)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
@@ -974,7 +982,7 @@
       <x:c r="D18" s="4"/>
       <x:c r="E18" s="4"/>
       <x:c r="F18" t="str">
-        <x:f>IF(COUNTA(A18:E18)=0,"",IF(OR(A18="",B18="",COUNTIFS($A$16:$A$35,A18)&gt;1,AND(C18&lt;&gt;"Ready",C18&lt;&gt;"Nonready",C18&lt;&gt;"Unknown"),AND(D18&lt;&gt;"Ready",D18&lt;&gt;"Not ready",D18&lt;&gt;"Unable to assess",D18&lt;&gt;"Missing",D18&lt;&gt;"")),"Invalid record",IF(B18&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A18:E18)=0,"",IF(OR(A18="",B18="",COUNTIFS($A$16:$A$35,A18)&gt;1,AND(C18&lt;&gt;"Ready",C18&lt;&gt;"Nonready",C18&lt;&gt;"Unknown"),AND(D18&lt;&gt;"Ready",D18&lt;&gt;"Not ready",D18&lt;&gt;"Unable to assess",D18&lt;&gt;"Missing",D18&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B18)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
@@ -984,7 +992,7 @@
       <x:c r="D19" s="4"/>
       <x:c r="E19" s="4"/>
       <x:c r="F19" t="str">
-        <x:f>IF(COUNTA(A19:E19)=0,"",IF(OR(A19="",B19="",COUNTIFS($A$16:$A$35,A19)&gt;1,AND(C19&lt;&gt;"Ready",C19&lt;&gt;"Nonready",C19&lt;&gt;"Unknown"),AND(D19&lt;&gt;"Ready",D19&lt;&gt;"Not ready",D19&lt;&gt;"Unable to assess",D19&lt;&gt;"Missing",D19&lt;&gt;"")),"Invalid record",IF(B19&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A19:E19)=0,"",IF(OR(A19="",B19="",COUNTIFS($A$16:$A$35,A19)&gt;1,AND(C19&lt;&gt;"Ready",C19&lt;&gt;"Nonready",C19&lt;&gt;"Unknown"),AND(D19&lt;&gt;"Ready",D19&lt;&gt;"Not ready",D19&lt;&gt;"Unable to assess",D19&lt;&gt;"Missing",D19&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B19)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
@@ -994,7 +1002,7 @@
       <x:c r="D20" s="4"/>
       <x:c r="E20" s="4"/>
       <x:c r="F20" t="str">
-        <x:f>IF(COUNTA(A20:E20)=0,"",IF(OR(A20="",B20="",COUNTIFS($A$16:$A$35,A20)&gt;1,AND(C20&lt;&gt;"Ready",C20&lt;&gt;"Nonready",C20&lt;&gt;"Unknown"),AND(D20&lt;&gt;"Ready",D20&lt;&gt;"Not ready",D20&lt;&gt;"Unable to assess",D20&lt;&gt;"Missing",D20&lt;&gt;"")),"Invalid record",IF(B20&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A20:E20)=0,"",IF(OR(A20="",B20="",COUNTIFS($A$16:$A$35,A20)&gt;1,AND(C20&lt;&gt;"Ready",C20&lt;&gt;"Nonready",C20&lt;&gt;"Unknown"),AND(D20&lt;&gt;"Ready",D20&lt;&gt;"Not ready",D20&lt;&gt;"Unable to assess",D20&lt;&gt;"Missing",D20&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B20)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
@@ -1004,7 +1012,7 @@
       <x:c r="D21" s="4"/>
       <x:c r="E21" s="4"/>
       <x:c r="F21" t="str">
-        <x:f>IF(COUNTA(A21:E21)=0,"",IF(OR(A21="",B21="",COUNTIFS($A$16:$A$35,A21)&gt;1,AND(C21&lt;&gt;"Ready",C21&lt;&gt;"Nonready",C21&lt;&gt;"Unknown"),AND(D21&lt;&gt;"Ready",D21&lt;&gt;"Not ready",D21&lt;&gt;"Unable to assess",D21&lt;&gt;"Missing",D21&lt;&gt;"")),"Invalid record",IF(B21&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A21:E21)=0,"",IF(OR(A21="",B21="",COUNTIFS($A$16:$A$35,A21)&gt;1,AND(C21&lt;&gt;"Ready",C21&lt;&gt;"Nonready",C21&lt;&gt;"Unknown"),AND(D21&lt;&gt;"Ready",D21&lt;&gt;"Not ready",D21&lt;&gt;"Unable to assess",D21&lt;&gt;"Missing",D21&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B21)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
@@ -1014,7 +1022,7 @@
       <x:c r="D22" s="4"/>
       <x:c r="E22" s="4"/>
       <x:c r="F22" t="str">
-        <x:f>IF(COUNTA(A22:E22)=0,"",IF(OR(A22="",B22="",COUNTIFS($A$16:$A$35,A22)&gt;1,AND(C22&lt;&gt;"Ready",C22&lt;&gt;"Nonready",C22&lt;&gt;"Unknown"),AND(D22&lt;&gt;"Ready",D22&lt;&gt;"Not ready",D22&lt;&gt;"Unable to assess",D22&lt;&gt;"Missing",D22&lt;&gt;"")),"Invalid record",IF(B22&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A22:E22)=0,"",IF(OR(A22="",B22="",COUNTIFS($A$16:$A$35,A22)&gt;1,AND(C22&lt;&gt;"Ready",C22&lt;&gt;"Nonready",C22&lt;&gt;"Unknown"),AND(D22&lt;&gt;"Ready",D22&lt;&gt;"Not ready",D22&lt;&gt;"Unable to assess",D22&lt;&gt;"Missing",D22&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B22)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
@@ -1024,7 +1032,7 @@
       <x:c r="D23" s="4"/>
       <x:c r="E23" s="4"/>
       <x:c r="F23" t="str">
-        <x:f>IF(COUNTA(A23:E23)=0,"",IF(OR(A23="",B23="",COUNTIFS($A$16:$A$35,A23)&gt;1,AND(C23&lt;&gt;"Ready",C23&lt;&gt;"Nonready",C23&lt;&gt;"Unknown"),AND(D23&lt;&gt;"Ready",D23&lt;&gt;"Not ready",D23&lt;&gt;"Unable to assess",D23&lt;&gt;"Missing",D23&lt;&gt;"")),"Invalid record",IF(B23&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A23:E23)=0,"",IF(OR(A23="",B23="",COUNTIFS($A$16:$A$35,A23)&gt;1,AND(C23&lt;&gt;"Ready",C23&lt;&gt;"Nonready",C23&lt;&gt;"Unknown"),AND(D23&lt;&gt;"Ready",D23&lt;&gt;"Not ready",D23&lt;&gt;"Unable to assess",D23&lt;&gt;"Missing",D23&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B23)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="24" ht="25" customHeight="1">
@@ -1034,7 +1042,7 @@
       <x:c r="D24" s="4"/>
       <x:c r="E24" s="4"/>
       <x:c r="F24" t="str">
-        <x:f>IF(COUNTA(A24:E24)=0,"",IF(OR(A24="",B24="",COUNTIFS($A$16:$A$35,A24)&gt;1,AND(C24&lt;&gt;"Ready",C24&lt;&gt;"Nonready",C24&lt;&gt;"Unknown"),AND(D24&lt;&gt;"Ready",D24&lt;&gt;"Not ready",D24&lt;&gt;"Unable to assess",D24&lt;&gt;"Missing",D24&lt;&gt;"")),"Invalid record",IF(B24&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A24:E24)=0,"",IF(OR(A24="",B24="",COUNTIFS($A$16:$A$35,A24)&gt;1,AND(C24&lt;&gt;"Ready",C24&lt;&gt;"Nonready",C24&lt;&gt;"Unknown"),AND(D24&lt;&gt;"Ready",D24&lt;&gt;"Not ready",D24&lt;&gt;"Unable to assess",D24&lt;&gt;"Missing",D24&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B24)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="25" ht="25" customHeight="1">
@@ -1044,7 +1052,7 @@
       <x:c r="D25" s="4"/>
       <x:c r="E25" s="4"/>
       <x:c r="F25" t="str">
-        <x:f>IF(COUNTA(A25:E25)=0,"",IF(OR(A25="",B25="",COUNTIFS($A$16:$A$35,A25)&gt;1,AND(C25&lt;&gt;"Ready",C25&lt;&gt;"Nonready",C25&lt;&gt;"Unknown"),AND(D25&lt;&gt;"Ready",D25&lt;&gt;"Not ready",D25&lt;&gt;"Unable to assess",D25&lt;&gt;"Missing",D25&lt;&gt;"")),"Invalid record",IF(B25&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A25:E25)=0,"",IF(OR(A25="",B25="",COUNTIFS($A$16:$A$35,A25)&gt;1,AND(C25&lt;&gt;"Ready",C25&lt;&gt;"Nonready",C25&lt;&gt;"Unknown"),AND(D25&lt;&gt;"Ready",D25&lt;&gt;"Not ready",D25&lt;&gt;"Unable to assess",D25&lt;&gt;"Missing",D25&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B25)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
@@ -1054,7 +1062,7 @@
       <x:c r="D26" s="4"/>
       <x:c r="E26" s="4"/>
       <x:c r="F26" t="str">
-        <x:f>IF(COUNTA(A26:E26)=0,"",IF(OR(A26="",B26="",COUNTIFS($A$16:$A$35,A26)&gt;1,AND(C26&lt;&gt;"Ready",C26&lt;&gt;"Nonready",C26&lt;&gt;"Unknown"),AND(D26&lt;&gt;"Ready",D26&lt;&gt;"Not ready",D26&lt;&gt;"Unable to assess",D26&lt;&gt;"Missing",D26&lt;&gt;"")),"Invalid record",IF(B26&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A26:E26)=0,"",IF(OR(A26="",B26="",COUNTIFS($A$16:$A$35,A26)&gt;1,AND(C26&lt;&gt;"Ready",C26&lt;&gt;"Nonready",C26&lt;&gt;"Unknown"),AND(D26&lt;&gt;"Ready",D26&lt;&gt;"Not ready",D26&lt;&gt;"Unable to assess",D26&lt;&gt;"Missing",D26&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B26)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
@@ -1064,7 +1072,7 @@
       <x:c r="D27" s="4"/>
       <x:c r="E27" s="4"/>
       <x:c r="F27" t="str">
-        <x:f>IF(COUNTA(A27:E27)=0,"",IF(OR(A27="",B27="",COUNTIFS($A$16:$A$35,A27)&gt;1,AND(C27&lt;&gt;"Ready",C27&lt;&gt;"Nonready",C27&lt;&gt;"Unknown"),AND(D27&lt;&gt;"Ready",D27&lt;&gt;"Not ready",D27&lt;&gt;"Unable to assess",D27&lt;&gt;"Missing",D27&lt;&gt;"")),"Invalid record",IF(B27&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A27:E27)=0,"",IF(OR(A27="",B27="",COUNTIFS($A$16:$A$35,A27)&gt;1,AND(C27&lt;&gt;"Ready",C27&lt;&gt;"Nonready",C27&lt;&gt;"Unknown"),AND(D27&lt;&gt;"Ready",D27&lt;&gt;"Not ready",D27&lt;&gt;"Unable to assess",D27&lt;&gt;"Missing",D27&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B27)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
@@ -1074,7 +1082,7 @@
       <x:c r="D28" s="4"/>
       <x:c r="E28" s="4"/>
       <x:c r="F28" t="str">
-        <x:f>IF(COUNTA(A28:E28)=0,"",IF(OR(A28="",B28="",COUNTIFS($A$16:$A$35,A28)&gt;1,AND(C28&lt;&gt;"Ready",C28&lt;&gt;"Nonready",C28&lt;&gt;"Unknown"),AND(D28&lt;&gt;"Ready",D28&lt;&gt;"Not ready",D28&lt;&gt;"Unable to assess",D28&lt;&gt;"Missing",D28&lt;&gt;"")),"Invalid record",IF(B28&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A28:E28)=0,"",IF(OR(A28="",B28="",COUNTIFS($A$16:$A$35,A28)&gt;1,AND(C28&lt;&gt;"Ready",C28&lt;&gt;"Nonready",C28&lt;&gt;"Unknown"),AND(D28&lt;&gt;"Ready",D28&lt;&gt;"Not ready",D28&lt;&gt;"Unable to assess",D28&lt;&gt;"Missing",D28&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B28)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
@@ -1084,7 +1092,7 @@
       <x:c r="D29" s="4"/>
       <x:c r="E29" s="4"/>
       <x:c r="F29" t="str">
-        <x:f>IF(COUNTA(A29:E29)=0,"",IF(OR(A29="",B29="",COUNTIFS($A$16:$A$35,A29)&gt;1,AND(C29&lt;&gt;"Ready",C29&lt;&gt;"Nonready",C29&lt;&gt;"Unknown"),AND(D29&lt;&gt;"Ready",D29&lt;&gt;"Not ready",D29&lt;&gt;"Unable to assess",D29&lt;&gt;"Missing",D29&lt;&gt;"")),"Invalid record",IF(B29&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A29:E29)=0,"",IF(OR(A29="",B29="",COUNTIFS($A$16:$A$35,A29)&gt;1,AND(C29&lt;&gt;"Ready",C29&lt;&gt;"Nonready",C29&lt;&gt;"Unknown"),AND(D29&lt;&gt;"Ready",D29&lt;&gt;"Not ready",D29&lt;&gt;"Unable to assess",D29&lt;&gt;"Missing",D29&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B29)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="30" ht="25" customHeight="1">
@@ -1094,7 +1102,7 @@
       <x:c r="D30" s="4"/>
       <x:c r="E30" s="4"/>
       <x:c r="F30" t="str">
-        <x:f>IF(COUNTA(A30:E30)=0,"",IF(OR(A30="",B30="",COUNTIFS($A$16:$A$35,A30)&gt;1,AND(C30&lt;&gt;"Ready",C30&lt;&gt;"Nonready",C30&lt;&gt;"Unknown"),AND(D30&lt;&gt;"Ready",D30&lt;&gt;"Not ready",D30&lt;&gt;"Unable to assess",D30&lt;&gt;"Missing",D30&lt;&gt;"")),"Invalid record",IF(B30&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A30:E30)=0,"",IF(OR(A30="",B30="",COUNTIFS($A$16:$A$35,A30)&gt;1,AND(C30&lt;&gt;"Ready",C30&lt;&gt;"Nonready",C30&lt;&gt;"Unknown"),AND(D30&lt;&gt;"Ready",D30&lt;&gt;"Not ready",D30&lt;&gt;"Unable to assess",D30&lt;&gt;"Missing",D30&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B30)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="31" ht="25" customHeight="1">
@@ -1104,7 +1112,7 @@
       <x:c r="D31" s="4"/>
       <x:c r="E31" s="4"/>
       <x:c r="F31" t="str">
-        <x:f>IF(COUNTA(A31:E31)=0,"",IF(OR(A31="",B31="",COUNTIFS($A$16:$A$35,A31)&gt;1,AND(C31&lt;&gt;"Ready",C31&lt;&gt;"Nonready",C31&lt;&gt;"Unknown"),AND(D31&lt;&gt;"Ready",D31&lt;&gt;"Not ready",D31&lt;&gt;"Unable to assess",D31&lt;&gt;"Missing",D31&lt;&gt;"")),"Invalid record",IF(B31&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A31:E31)=0,"",IF(OR(A31="",B31="",COUNTIFS($A$16:$A$35,A31)&gt;1,AND(C31&lt;&gt;"Ready",C31&lt;&gt;"Nonready",C31&lt;&gt;"Unknown"),AND(D31&lt;&gt;"Ready",D31&lt;&gt;"Not ready",D31&lt;&gt;"Unable to assess",D31&lt;&gt;"Missing",D31&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B31)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="32" ht="25" customHeight="1">
@@ -1114,7 +1122,7 @@
       <x:c r="D32" s="4"/>
       <x:c r="E32" s="4"/>
       <x:c r="F32" t="str">
-        <x:f>IF(COUNTA(A32:E32)=0,"",IF(OR(A32="",B32="",COUNTIFS($A$16:$A$35,A32)&gt;1,AND(C32&lt;&gt;"Ready",C32&lt;&gt;"Nonready",C32&lt;&gt;"Unknown"),AND(D32&lt;&gt;"Ready",D32&lt;&gt;"Not ready",D32&lt;&gt;"Unable to assess",D32&lt;&gt;"Missing",D32&lt;&gt;"")),"Invalid record",IF(B32&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A32:E32)=0,"",IF(OR(A32="",B32="",COUNTIFS($A$16:$A$35,A32)&gt;1,AND(C32&lt;&gt;"Ready",C32&lt;&gt;"Nonready",C32&lt;&gt;"Unknown"),AND(D32&lt;&gt;"Ready",D32&lt;&gt;"Not ready",D32&lt;&gt;"Unable to assess",D32&lt;&gt;"Missing",D32&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B32)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="33" ht="25" customHeight="1">
@@ -1124,7 +1132,7 @@
       <x:c r="D33" s="4"/>
       <x:c r="E33" s="4"/>
       <x:c r="F33" t="str">
-        <x:f>IF(COUNTA(A33:E33)=0,"",IF(OR(A33="",B33="",COUNTIFS($A$16:$A$35,A33)&gt;1,AND(C33&lt;&gt;"Ready",C33&lt;&gt;"Nonready",C33&lt;&gt;"Unknown"),AND(D33&lt;&gt;"Ready",D33&lt;&gt;"Not ready",D33&lt;&gt;"Unable to assess",D33&lt;&gt;"Missing",D33&lt;&gt;"")),"Invalid record",IF(B33&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A33:E33)=0,"",IF(OR(A33="",B33="",COUNTIFS($A$16:$A$35,A33)&gt;1,AND(C33&lt;&gt;"Ready",C33&lt;&gt;"Nonready",C33&lt;&gt;"Unknown"),AND(D33&lt;&gt;"Ready",D33&lt;&gt;"Not ready",D33&lt;&gt;"Unable to assess",D33&lt;&gt;"Missing",D33&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B33)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="34" ht="25" customHeight="1">
@@ -1134,7 +1142,7 @@
       <x:c r="D34" s="4"/>
       <x:c r="E34" s="4"/>
       <x:c r="F34" t="str">
-        <x:f>IF(COUNTA(A34:E34)=0,"",IF(OR(A34="",B34="",COUNTIFS($A$16:$A$35,A34)&gt;1,AND(C34&lt;&gt;"Ready",C34&lt;&gt;"Nonready",C34&lt;&gt;"Unknown"),AND(D34&lt;&gt;"Ready",D34&lt;&gt;"Not ready",D34&lt;&gt;"Unable to assess",D34&lt;&gt;"Missing",D34&lt;&gt;"")),"Invalid record",IF(B34&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A34:E34)=0,"",IF(OR(A34="",B34="",COUNTIFS($A$16:$A$35,A34)&gt;1,AND(C34&lt;&gt;"Ready",C34&lt;&gt;"Nonready",C34&lt;&gt;"Unknown"),AND(D34&lt;&gt;"Ready",D34&lt;&gt;"Not ready",D34&lt;&gt;"Unable to assess",D34&lt;&gt;"Missing",D34&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B34)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="35" ht="25" customHeight="1">
@@ -1144,7 +1152,7 @@
       <x:c r="D35" s="4"/>
       <x:c r="E35" s="4"/>
       <x:c r="F35" t="str">
-        <x:f>IF(COUNTA(A35:E35)=0,"",IF(OR(A35="",B35="",COUNTIFS($A$16:$A$35,A35)&gt;1,AND(C35&lt;&gt;"Ready",C35&lt;&gt;"Nonready",C35&lt;&gt;"Unknown"),AND(D35&lt;&gt;"Ready",D35&lt;&gt;"Not ready",D35&lt;&gt;"Unable to assess",D35&lt;&gt;"Missing",D35&lt;&gt;"")),"Invalid record",IF(B35&lt;&gt;$B$16,"Mixed criteria","Valid")))</x:f>
+        <x:f>IF(COUNTA(A35:E35)=0,"",IF(OR(A35="",B35="",COUNTIFS($A$16:$A$35,A35)&gt;1,AND(C35&lt;&gt;"Ready",C35&lt;&gt;"Nonready",C35&lt;&gt;"Unknown"),AND(D35&lt;&gt;"Ready",D35&lt;&gt;"Not ready",D35&lt;&gt;"Unable to assess",D35&lt;&gt;"Missing",D35&lt;&gt;"")),"Invalid record",IF(COUNTIFS($B$16:$B$35,B35)&lt;&gt;COUNTIFS($A$16:$A$35,"&lt;&gt;"),"Mixed criteria","Valid")))</x:f>
       </x:c>
     </x:row>
     <x:row r="36" ht="25" customHeight="1">
@@ -1161,12 +1169,103 @@
       <x:c r="D37" s="2"/>
       <x:c r="E37" s="2"/>
     </x:row>
-    <x:row r="38" ht="25" customHeight="1">
-      <x:c r="A38" s="2"/>
-      <x:c r="B38" s="2"/>
+    <x:row r="38" ht="28" customHeight="1">
+      <x:c r="A38" s="10" t="str">
+        <x:v>Companion measures</x:v>
+      </x:c>
+      <x:c r="B38" s="10" t="str">
+        <x:v>Result</x:v>
+      </x:c>
       <x:c r="C38" s="2"/>
       <x:c r="D38" s="2"/>
       <x:c r="E38" s="2"/>
+      <x:c r="F38" s="1"/>
+    </x:row>
+    <x:row r="39" ht="28" customHeight="1">
+      <x:c r="A39" s="1" t="str">
+        <x:v>Decision coverage on nonready instances</x:v>
+      </x:c>
+      <x:c r="B39" s="13" t="str">
+        <x:f>IF(NOT(ISNUMBER(B5)),"Not evaluated",IF(B5=0,"n.a.",(B5-B7)/B5))</x:f>
+        <x:v>Not evaluated</x:v>
+      </x:c>
+      <x:c r="C39" s="1" t="str">
+        <x:v>(Ready + Not ready) / all observed Nonready judgments.</x:v>
+      </x:c>
+      <x:c r="D39" s="1"/>
+      <x:c r="E39" s="1"/>
+      <x:c r="F39" s="1"/>
+    </x:row>
+    <x:row r="40" ht="28" customHeight="1">
+      <x:c r="A40" s="1" t="str">
+        <x:v>False-ready among decisive judgments</x:v>
+      </x:c>
+      <x:c r="B40" s="13" t="str">
+        <x:f>IF(NOT(ISNUMBER(B5)),"Not evaluated",IF(B5-B7=0,"n.a.",B6/(B5-B7)))</x:f>
+        <x:v>Not evaluated</x:v>
+      </x:c>
+      <x:c r="C40" s="1" t="str">
+        <x:v>Ready / (Ready + Not ready) on Nonready artifacts.</x:v>
+      </x:c>
+      <x:c r="D40" s="1"/>
+      <x:c r="E40" s="1"/>
+      <x:c r="F40" s="1"/>
+    </x:row>
+    <x:row r="41" ht="28" customHeight="1">
+      <x:c r="A41" s="1" t="str">
+        <x:v>Ready instances with observed judgment</x:v>
+      </x:c>
+      <x:c r="B41" s="1" t="str">
+        <x:f>IF(B12&lt;&gt;"Valid","Not evaluated",COUNTIFS(C16:C35,"Ready",D16:D35,"Ready")+COUNTIFS(C16:C35,"Ready",D16:D35,"Not ready")+COUNTIFS(C16:C35,"Ready",D16:D35,"Unable to assess"))</x:f>
+        <x:v>Not evaluated</x:v>
+      </x:c>
+      <x:c r="C41" s="1"/>
+      <x:c r="D41" s="1"/>
+      <x:c r="E41" s="1"/>
+      <x:c r="F41" s="1"/>
+    </x:row>
+    <x:row r="42" ht="28" customHeight="1">
+      <x:c r="A42" s="1" t="str">
+        <x:v>False hold rate on ready instances</x:v>
+      </x:c>
+      <x:c r="B42" s="13" t="str">
+        <x:f>IF(NOT(ISNUMBER(B41)),"Not evaluated",IF(B41=0,"n.a.",COUNTIFS(C16:C35,"Ready",D16:D35,"Not ready")/B41))</x:f>
+        <x:v>Not evaluated</x:v>
+      </x:c>
+      <x:c r="C42" s="1" t="str">
+        <x:v>Not ready / all observed judgments on Ready artifacts.</x:v>
+      </x:c>
+      <x:c r="D42" s="1"/>
+      <x:c r="E42" s="1"/>
+      <x:c r="F42" s="1"/>
+    </x:row>
+    <x:row r="43" ht="28" customHeight="1">
+      <x:c r="A43" s="1" t="str">
+        <x:v>Abstention rate on ready instances</x:v>
+      </x:c>
+      <x:c r="B43" s="13" t="str">
+        <x:f>IF(NOT(ISNUMBER(B41)),"Not evaluated",IF(B41=0,"n.a.",COUNTIFS(C16:C35,"Ready",D16:D35,"Unable to assess")/B41))</x:f>
+        <x:v>Not evaluated</x:v>
+      </x:c>
+      <x:c r="C43" s="1" t="str">
+        <x:v>Report alongside false hold; never infer usefulness from one rate.</x:v>
+      </x:c>
+      <x:c r="D43" s="1"/>
+      <x:c r="E43" s="1"/>
+      <x:c r="F43" s="1"/>
+    </x:row>
+    <x:row r="44" ht="28" customHeight="1">
+      <x:c r="A44" s="1" t="str">
+        <x:v>Missing judgments on ready instances</x:v>
+      </x:c>
+      <x:c r="B44" s="1" t="str">
+        <x:f>IF(B12&lt;&gt;"Valid","Not evaluated",COUNTIFS(C16:C35,"Ready")-B41)</x:f>
+        <x:v>Not evaluated</x:v>
+      </x:c>
+      <x:c r="C44" s="1"/>
+      <x:c r="D44" s="1"/>
+      <x:c r="E44" s="1"/>
+      <x:c r="F44" s="1"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F16:F35">

</xml_diff>